<commit_message>
docs: No ocurrio nada (sin relevancia)
</commit_message>
<xml_diff>
--- a/proyectos_diseno/BASES_DE_DATOS/Festivos.xlsx
+++ b/proyectos_diseno/BASES_DE_DATOS/Festivos.xlsx
@@ -10,7 +10,7 @@
     <sheet name="FESTIVOS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FESTIVOS'!$A$1:$E$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FESTIVOS'!$A$1:$E$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -147,8 +147,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TB_FESTIVOS" displayName="TB_FESTIVOS" ref="A1:E39" headerRowCount="1">
-  <autoFilter ref="A1:E39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TB_FESTIVOS" displayName="TB_FESTIVOS" ref="A1:E56" headerRowCount="1">
+  <autoFilter ref="A1:E56"/>
   <tableColumns count="5">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="fecha"/>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1436,8 +1436,433 @@
         <v>1</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2da9a3c5-5a54-4e41-a277-de417438b5b0</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Año Nuevo</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>45273070-2533-4381-891a-c45e1e86b808</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>2025-01-06</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Día de los Reyes Magos</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>a93e1c1a-061f-4a36-904e-daeecba485b1</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>2025-03-24</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Día de San José (observado)</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>75e5eaaf-07b9-447b-b4cb-0787bb3ff603</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>2025-04-17</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Jueves Santo</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>9ede084a-96e2-454c-9e76-3487f397b91f</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2025-04-18</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Viernes Santo</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>f3aaca68-e8be-4fef-85d0-866c99af0ade</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Día del Trabajo</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>cd4b6837-5f86-45ee-9766-76a23a0a4c01</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-02</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Ascensión del señor (observado)</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>f81959c5-df96-48b7-8f37-f6e90bfd3e49</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-23</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Corpus Christi (observado)</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>524081dd-e739-41c2-b10f-5f9b4acb54b0</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Sagrado Corazón (observado); San Pedro y San Pablo (observado)</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>7919702a-b8e1-4050-93c1-986d01406f0f</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2025-07-20</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Día de la Independencia</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>d5a81bba-72e3-443c-bfd1-8b43279fc50a</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2025-08-07</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Batalla de Boyacá</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>a3d342ee-fdb8-480c-8f93-dab91dd68b87</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>2025-08-18</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>La Asunción (observado)</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>a554118f-fa8b-4b63-b6c8-1c57712683bc</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>2025-10-13</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Día de la Raza (observado)</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>b302654c-b818-437a-8ce2-68ef0fd29932</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Día de Todos los Santos (observado)</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>c0f4dd54-33cb-4262-a515-ea1ede9f55b5</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-17</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Independencia de Cartagena (observado)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>6d0bb88d-598b-4fc2-9513-d1f481b48beb</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>La Inmaculada Concepción</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>b5ae538b-3c72-48e9-830a-7c8a775ca06f</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Navidad</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Colombia automático</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E39"/>
+  <autoFilter ref="A1:E56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>